<commit_message>
feat: verify rule CG0061 and add negative test cases
</commit_message>
<xml_diff>
--- a/rules/CORE-000257/negative/01/data/unit-test-coreid-CG0061-negative 1.xlsx
+++ b/rules/CORE-000257/negative/01/data/unit-test-coreid-CG0061-negative 1.xlsx
@@ -35,7 +35,7 @@
       <i val="1"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -52,6 +52,12 @@
       <patternFill patternType="solid">
         <fgColor theme="0" tint="-0.1499984740745262"/>
         <bgColor theme="0" tint="-0.1499984740745262"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor rgb="FFFFFF00"/>
       </patternFill>
     </fill>
   </fills>
@@ -82,7 +88,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -105,6 +111,9 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -548,7 +557,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:F13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -580,6 +589,312 @@
       <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Error value</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>pr.xpt</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>5</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>PRSTRTPT</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>AFTER</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>pr.xpt</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>5</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>PRSTTPT</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>2</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>pr.xpt</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>6</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>PRSTRTPT</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>AFTER</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>2</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>pr.xpt</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>6</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>PRSTTPT</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>3</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>pr.xpt</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>7</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>PRSTRTPT</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>AFTER</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>3</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>pr.xpt</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>7</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>PRSTTPT</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>4</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>pr.xpt</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>8</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>PRSTRTPT</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>BEFORE</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>4</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>pr.xpt</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>8</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>PRSTTPT</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>5</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>pr.xpt</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>9</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>PRSTRTPT</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>BEFORE</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>5</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>pr.xpt</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>9</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>PRSTTPT</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>6</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>pr.xpt</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>10</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>PRSTRTPT</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>BEFORE</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>6</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>pr.xpt</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>10</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>PRSTTPT</t>
         </is>
       </c>
     </row>
@@ -1085,12 +1400,12 @@
       <c r="S5" s="7" t="n">
         <v>111</v>
       </c>
-      <c r="T5" s="6" t="inlineStr">
+      <c r="T5" s="10" t="inlineStr">
         <is>
           <t>AFTER</t>
         </is>
       </c>
-      <c r="U5" s="6" t="n"/>
+      <c r="U5" s="10" t="n"/>
       <c r="V5" s="6" t="n"/>
       <c r="W5" s="6" t="n"/>
     </row>
@@ -1162,12 +1477,12 @@
       <c r="S6" s="9" t="n">
         <v>117</v>
       </c>
-      <c r="T6" s="8" t="inlineStr">
+      <c r="T6" s="10" t="inlineStr">
         <is>
           <t>AFTER</t>
         </is>
       </c>
-      <c r="U6" s="8" t="n"/>
+      <c r="U6" s="10" t="n"/>
       <c r="V6" s="8" t="n"/>
       <c r="W6" s="8" t="n"/>
     </row>
@@ -1237,12 +1552,12 @@
       <c r="S7" s="7" t="n">
         <v>117</v>
       </c>
-      <c r="T7" s="6" t="inlineStr">
+      <c r="T7" s="10" t="inlineStr">
         <is>
           <t>AFTER</t>
         </is>
       </c>
-      <c r="U7" s="6" t="n"/>
+      <c r="U7" s="10" t="n"/>
       <c r="V7" s="6" t="n"/>
       <c r="W7" s="6" t="n"/>
     </row>
@@ -1322,12 +1637,12 @@
         <v>1</v>
       </c>
       <c r="S8" s="8" t="n"/>
-      <c r="T8" s="8" t="inlineStr">
+      <c r="T8" s="10" t="inlineStr">
         <is>
           <t>BEFORE</t>
         </is>
       </c>
-      <c r="U8" s="8" t="n"/>
+      <c r="U8" s="10" t="n"/>
       <c r="V8" s="8" t="n"/>
       <c r="W8" s="8" t="n"/>
     </row>
@@ -1397,12 +1712,12 @@
       <c r="S9" s="7" t="n">
         <v>23</v>
       </c>
-      <c r="T9" s="6" t="inlineStr">
+      <c r="T9" s="10" t="inlineStr">
         <is>
           <t>BEFORE</t>
         </is>
       </c>
-      <c r="U9" s="6" t="n"/>
+      <c r="U9" s="10" t="n"/>
       <c r="V9" s="6" t="n"/>
       <c r="W9" s="6" t="n"/>
     </row>
@@ -1474,12 +1789,12 @@
       <c r="S10" s="9" t="n">
         <v>28</v>
       </c>
-      <c r="T10" s="8" t="inlineStr">
+      <c r="T10" s="10" t="inlineStr">
         <is>
           <t>BEFORE</t>
         </is>
       </c>
-      <c r="U10" s="8" t="n"/>
+      <c r="U10" s="10" t="n"/>
       <c r="V10" s="8" t="n"/>
       <c r="W10" s="8" t="n"/>
     </row>

</xml_diff>